<commit_message>
Update DMC System: 2026-09-16 10:48:53.22
</commit_message>
<xml_diff>
--- a/Excel/M-0.xlsx
+++ b/Excel/M-0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dara1\OneDrive\Desktop\DCM_System\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F467BCD4-C54B-4E8E-816E-325CFA8357AC}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713A4B6A-75EC-4FE0-92C7-E4746B820665}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A1E7FE79-11C2-4822-9E17-1FEC213DBAB3}"/>
   </bookViews>
@@ -553,30 +553,9 @@
   </cellStyleXfs>
   <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -587,15 +566,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -628,6 +598,36 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1755,1879 +1755,1891 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.5" x14ac:dyDescent="0.7">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="A1" s="23"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:10" ht="25.5" x14ac:dyDescent="0.7">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
     </row>
     <row r="3" spans="1:10" ht="30.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
     </row>
     <row r="4" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="5"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
     </row>
     <row r="6" spans="1:10" ht="5.25" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
     </row>
     <row r="7" spans="1:10" ht="23.25" x14ac:dyDescent="0.65">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
     </row>
     <row r="8" spans="1:10" ht="23.25" x14ac:dyDescent="0.65">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
     </row>
     <row r="9" spans="1:10" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="G9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
     </row>
     <row r="10" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-    </row>
-    <row r="11" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17">
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7">
         <v>1</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="20" t="s">
+      <c r="C11" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="19" t="s">
+      <c r="H11" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17">
+    <row r="12" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
         <v>2</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="20" t="s">
+      <c r="C12" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="21" t="s">
+      <c r="F12" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H12" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="22" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17">
+    <row r="13" spans="1:10" s="12" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="7">
         <v>3</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" s="20" t="s">
+      <c r="C13" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10" t="s">
+      <c r="H13" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17">
+    <row r="14" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7">
         <v>4</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="20" t="s">
+      <c r="C14" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H14" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J14" s="10" t="s">
+      <c r="H14" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
+    <row r="15" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7">
         <v>5</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="20" t="s">
+      <c r="C15" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="19" t="s">
+      <c r="E15" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H15" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
+      <c r="H15" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7">
         <v>6</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D16" s="20" t="s">
+      <c r="C16" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H16" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17">
+      <c r="H16" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7">
         <v>7</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D17" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E17" s="19" t="s">
+      <c r="E17" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I17" s="23"/>
-    </row>
-    <row r="18" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17">
+      <c r="H17" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="13"/>
+    </row>
+    <row r="18" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7">
         <v>8</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="G18" s="19" t="s">
+      <c r="G18" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="H18" s="19"/>
+      <c r="H18" s="9"/>
     </row>
     <row r="19" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-    </row>
-    <row r="20" spans="1:10" s="22" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17">
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" spans="1:10" s="12" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="7">
         <v>1</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D20" s="20" t="s">
+      <c r="C20" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E20" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="19" t="s">
+      <c r="F20" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G20" s="19" t="s">
+      <c r="G20" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H20" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-    </row>
-    <row r="21" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17">
+      <c r="H20" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+    </row>
+    <row r="21" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7">
         <v>2</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" s="20" t="s">
+      <c r="C21" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="F21" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H21" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17">
+      <c r="H21" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7">
         <v>3</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D22" s="20" t="s">
+      <c r="C22" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="E22" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H22" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I22" s="24" t="s">
+      <c r="H22" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I22" s="14" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="17">
+    <row r="23" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="7">
         <v>4</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D23" s="20" t="s">
+      <c r="C23" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="E23" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F23" s="19" t="s">
+      <c r="F23" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G23" s="19" t="s">
+      <c r="G23" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H23" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I23" s="24"/>
-    </row>
-    <row r="24" spans="1:10" s="22" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="17">
+      <c r="H23" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I23" s="14"/>
+    </row>
+    <row r="24" spans="1:10" s="12" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="7">
         <v>5</v>
       </c>
-      <c r="B24" s="25" t="s">
+      <c r="B24" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D24" s="20" t="s">
+      <c r="C24" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F24" s="19" t="s">
+      <c r="F24" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H24" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I24" s="24"/>
-      <c r="J24" s="10"/>
-    </row>
-    <row r="25" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="17">
+      <c r="H24" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I24" s="14"/>
+      <c r="J24" s="3"/>
+    </row>
+    <row r="25" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="7">
         <v>6</v>
       </c>
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D25" s="20" t="s">
+      <c r="C25" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E25" s="19" t="s">
+      <c r="E25" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F25" s="19" t="s">
+      <c r="F25" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H25" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I25" s="24" t="s">
+      <c r="H25" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I25" s="14" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="17">
+    <row r="26" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="7">
         <v>7</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D26" s="20" t="s">
+      <c r="C26" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="19" t="s">
+      <c r="E26" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F26" s="19" t="s">
+      <c r="F26" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G26" s="19" t="s">
+      <c r="G26" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H26" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="17">
+      <c r="H26" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="7">
         <v>8</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C27" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" s="20" t="s">
+      <c r="C27" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F27" s="19" t="s">
+      <c r="F27" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H27" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="17">
+      <c r="H27" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="7">
         <v>9</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C28" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" s="28" t="s">
+      <c r="C28" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="E28" s="19" t="s">
+      <c r="E28" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F28" s="19" t="s">
+      <c r="F28" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G28" s="19" t="s">
+      <c r="G28" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H28" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I28" s="24"/>
-    </row>
-    <row r="29" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="17">
+      <c r="H28" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I28" s="14"/>
+    </row>
+    <row r="29" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="7">
         <v>10</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D29" s="20" t="s">
+      <c r="C29" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E29" s="19" t="s">
+      <c r="E29" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="F29" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G29" s="19" t="s">
+      <c r="G29" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H29" s="19" t="s">
+      <c r="H29" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-    </row>
-    <row r="31" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="17">
+      <c r="B30" s="20"/>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+    </row>
+    <row r="31" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="7">
         <v>1</v>
       </c>
-      <c r="B31" s="18" t="s">
+      <c r="B31" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D31" s="20" t="s">
+      <c r="C31" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E31" s="19" t="s">
+      <c r="E31" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F31" s="19" t="s">
+      <c r="F31" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G31" s="19" t="s">
+      <c r="G31" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H31" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="17">
+      <c r="H31" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="7">
         <v>2</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D32" s="20" t="s">
+      <c r="C32" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E32" s="19" t="s">
+      <c r="E32" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F32" s="19" t="s">
+      <c r="F32" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G32" s="19" t="s">
+      <c r="G32" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H32" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="17">
+      <c r="H32" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="7">
         <v>3</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D33" s="20" t="s">
+      <c r="C33" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E33" s="19" t="s">
+      <c r="E33" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F33" s="19" t="s">
+      <c r="F33" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G33" s="19" t="s">
+      <c r="G33" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H33" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="17">
+      <c r="H33" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="7">
         <v>4</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B34" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C34" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" s="20" t="s">
+      <c r="C34" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E34" s="19" t="s">
+      <c r="E34" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F34" s="19" t="s">
+      <c r="F34" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="G34" s="19" t="s">
+      <c r="G34" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H34" s="19" t="s">
+      <c r="H34" s="9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="17">
+    <row r="35" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="7">
         <v>5</v>
       </c>
-      <c r="B35" s="18" t="s">
+      <c r="B35" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C35" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D35" s="20" t="s">
+      <c r="C35" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E35" s="19" t="s">
+      <c r="E35" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F35" s="19" t="s">
+      <c r="F35" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G35" s="19" t="s">
+      <c r="G35" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H35" s="19" t="s">
+      <c r="H35" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
+      <c r="A36" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15"/>
-      <c r="F36" s="15"/>
-      <c r="G36" s="15"/>
-      <c r="H36" s="16"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
-    </row>
-    <row r="37" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="17">
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+    </row>
+    <row r="37" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="7">
         <v>1</v>
       </c>
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C37" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D37" s="20" t="s">
+      <c r="C37" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E37" s="19" t="s">
+      <c r="E37" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F37" s="19" t="s">
+      <c r="F37" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G37" s="19" t="s">
+      <c r="G37" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H37" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="17">
+      <c r="H37" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="7">
         <v>2</v>
       </c>
-      <c r="B38" s="18" t="s">
+      <c r="B38" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C38" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D38" s="20" t="s">
+      <c r="C38" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E38" s="19" t="s">
+      <c r="E38" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F38" s="19" t="s">
+      <c r="F38" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="G38" s="19" t="s">
+      <c r="G38" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H38" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I38" s="10">
+      <c r="H38" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I38" s="3">
         <v>2023</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
+      <c r="A39" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="B39" s="15"/>
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="15"/>
-      <c r="F39" s="15"/>
-      <c r="G39" s="15"/>
-      <c r="H39" s="16"/>
-      <c r="I39" s="10"/>
-      <c r="J39" s="10"/>
-    </row>
-    <row r="40" spans="1:10" s="22" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="17">
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="20"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+    </row>
+    <row r="40" spans="1:10" s="12" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="7">
         <v>1</v>
       </c>
-      <c r="B40" s="18" t="s">
+      <c r="B40" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="C40" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D40" s="20" t="s">
+      <c r="C40" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E40" s="19" t="s">
+      <c r="E40" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F40" s="19" t="s">
+      <c r="F40" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G40" s="19" t="s">
+      <c r="G40" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H40" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I40" s="10"/>
-      <c r="J40" s="10" t="s">
+      <c r="H40" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="17">
+    <row r="41" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="7">
         <v>2</v>
       </c>
-      <c r="B41" s="18" t="s">
+      <c r="B41" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="C41" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D41" s="20" t="s">
+      <c r="C41" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D41" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E41" s="19" t="s">
+      <c r="E41" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F41" s="19" t="s">
+      <c r="F41" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="G41" s="19" t="s">
+      <c r="G41" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H41" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J41" s="10" t="s">
+      <c r="H41" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J41" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="42" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="17">
+    <row r="42" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="7">
         <v>3</v>
       </c>
-      <c r="B42" s="18" t="s">
+      <c r="B42" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C42" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D42" s="20" t="s">
+      <c r="C42" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E42" s="19" t="s">
+      <c r="E42" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F42" s="19" t="s">
+      <c r="F42" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G42" s="19" t="s">
+      <c r="G42" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H42" s="19" t="s">
+      <c r="H42" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
+      <c r="A43" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="B43" s="15"/>
-      <c r="C43" s="15"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="16"/>
-      <c r="I43" s="10"/>
-      <c r="J43" s="10"/>
-    </row>
-    <row r="44" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="17">
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="21"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+    </row>
+    <row r="44" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="7">
         <v>1</v>
       </c>
-      <c r="B44" s="18" t="s">
+      <c r="B44" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C44" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D44" s="20" t="s">
+      <c r="C44" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E44" s="19" t="s">
+      <c r="E44" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F44" s="19" t="s">
+      <c r="F44" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="G44" s="19" t="s">
+      <c r="G44" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H44" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I44" s="10">
+      <c r="H44" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I44" s="3">
         <v>2023</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="17">
+      <c r="A45" s="7">
         <v>2</v>
       </c>
-      <c r="B45" s="18" t="s">
+      <c r="B45" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C45" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D45" s="20" t="s">
+      <c r="C45" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E45" s="19" t="s">
+      <c r="E45" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F45" s="19" t="s">
+      <c r="F45" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G45" s="19" t="s">
+      <c r="G45" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H45" s="19" t="s">
+      <c r="H45" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="I45" s="10"/>
-      <c r="J45" s="10"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
     </row>
     <row r="46" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="14" t="s">
+      <c r="A46" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B46" s="15"/>
-      <c r="C46" s="15"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15"/>
-      <c r="F46" s="15"/>
-      <c r="G46" s="15"/>
-      <c r="H46" s="16"/>
-      <c r="I46" s="10"/>
-      <c r="J46" s="10"/>
-    </row>
-    <row r="47" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="17">
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
+      <c r="H46" s="21"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+    </row>
+    <row r="47" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="7">
         <v>1</v>
       </c>
-      <c r="B47" s="18" t="s">
+      <c r="B47" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C47" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D47" s="20" t="s">
+      <c r="C47" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E47" s="19" t="s">
+      <c r="E47" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F47" s="19" t="s">
+      <c r="F47" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="G47" s="19" t="s">
+      <c r="G47" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H47" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I47" s="10">
+      <c r="H47" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I47" s="3">
         <v>2023</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
+      <c r="A48" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="15"/>
-      <c r="C48" s="15"/>
-      <c r="D48" s="15"/>
-      <c r="E48" s="15"/>
-      <c r="F48" s="15"/>
-      <c r="G48" s="15"/>
-      <c r="H48" s="16"/>
-      <c r="I48" s="10"/>
-      <c r="J48" s="10"/>
-    </row>
-    <row r="49" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="17">
+      <c r="B48" s="20"/>
+      <c r="C48" s="20"/>
+      <c r="D48" s="20"/>
+      <c r="E48" s="20"/>
+      <c r="F48" s="20"/>
+      <c r="G48" s="20"/>
+      <c r="H48" s="21"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+    </row>
+    <row r="49" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="7">
         <v>1</v>
       </c>
-      <c r="B49" s="18" t="s">
+      <c r="B49" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C49" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D49" s="20" t="s">
+      <c r="C49" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D49" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E49" s="19" t="s">
+      <c r="E49" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F49" s="19" t="s">
+      <c r="F49" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="G49" s="19" t="s">
+      <c r="G49" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H49" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I49" s="10">
+      <c r="H49" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I49" s="3">
         <v>2023</v>
       </c>
     </row>
-    <row r="50" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="17">
+    <row r="50" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="7">
         <v>2</v>
       </c>
-      <c r="B50" s="18" t="s">
+      <c r="B50" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C50" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D50" s="20" t="s">
+      <c r="C50" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D50" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E50" s="19" t="s">
+      <c r="E50" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F50" s="19" t="s">
+      <c r="F50" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="G50" s="19" t="s">
+      <c r="G50" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H50" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="17">
+      <c r="H50" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="7">
         <v>3</v>
       </c>
-      <c r="B51" s="18" t="s">
+      <c r="B51" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="C51" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D51" s="20" t="s">
+      <c r="C51" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D51" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E51" s="19" t="s">
+      <c r="E51" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F51" s="19" t="s">
+      <c r="F51" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="G51" s="19" t="s">
+      <c r="G51" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H51" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="17">
+      <c r="H51" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="7">
         <v>4</v>
       </c>
-      <c r="B52" s="18" t="s">
+      <c r="B52" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="C52" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D52" s="20" t="s">
+      <c r="C52" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D52" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E52" s="19" t="s">
+      <c r="E52" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F52" s="19" t="s">
+      <c r="F52" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G52" s="19" t="s">
+      <c r="G52" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H52" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="17">
+      <c r="H52" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="7">
         <v>5</v>
       </c>
-      <c r="B53" s="18" t="s">
+      <c r="B53" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="C53" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D53" s="20" t="s">
+      <c r="C53" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D53" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E53" s="19" t="s">
+      <c r="E53" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F53" s="19" t="s">
+      <c r="F53" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="G53" s="19" t="s">
+      <c r="G53" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H53" s="19" t="s">
+      <c r="H53" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="14" t="s">
+      <c r="A54" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B54" s="15"/>
-      <c r="C54" s="15"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="15"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="16"/>
-      <c r="I54" s="10"/>
-      <c r="J54" s="10"/>
-    </row>
-    <row r="55" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="17">
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
+      <c r="E54" s="20"/>
+      <c r="F54" s="20"/>
+      <c r="G54" s="20"/>
+      <c r="H54" s="21"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+    </row>
+    <row r="55" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="7">
         <v>1</v>
       </c>
-      <c r="B55" s="18" t="s">
+      <c r="B55" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="C55" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D55" s="20" t="s">
+      <c r="C55" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D55" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E55" s="19" t="s">
+      <c r="E55" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F55" s="19" t="s">
+      <c r="F55" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="G55" s="19" t="s">
+      <c r="G55" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H55" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="17">
+      <c r="H55" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="7">
         <v>2</v>
       </c>
-      <c r="B56" s="18" t="s">
+      <c r="B56" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="C56" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D56" s="20" t="s">
+      <c r="C56" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D56" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E56" s="19" t="s">
+      <c r="E56" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F56" s="19" t="s">
+      <c r="F56" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="G56" s="19" t="s">
+      <c r="G56" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H56" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="17">
+      <c r="H56" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="7">
         <v>3</v>
       </c>
-      <c r="B57" s="18" t="s">
+      <c r="B57" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="C57" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D57" s="20" t="s">
+      <c r="C57" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D57" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E57" s="19" t="s">
+      <c r="E57" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F57" s="19" t="s">
+      <c r="F57" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G57" s="19" t="s">
+      <c r="G57" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H57" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="17">
+      <c r="H57" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="7">
         <v>4</v>
       </c>
-      <c r="B58" s="18" t="s">
+      <c r="B58" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="C58" s="19" t="s">
+      <c r="C58" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D58" s="20" t="s">
+      <c r="D58" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E58" s="19" t="s">
+      <c r="E58" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F58" s="19" t="s">
+      <c r="F58" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G58" s="19" t="s">
+      <c r="G58" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H58" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="17">
+      <c r="H58" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="7">
         <v>5</v>
       </c>
-      <c r="B59" s="18" t="s">
+      <c r="B59" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="C59" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D59" s="20" t="s">
+      <c r="C59" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D59" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E59" s="19" t="s">
+      <c r="E59" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F59" s="19" t="s">
+      <c r="F59" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="G59" s="19" t="s">
+      <c r="G59" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H59" s="19" t="s">
+      <c r="H59" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="14" t="s">
+      <c r="A60" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="B60" s="15"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="15"/>
-      <c r="F60" s="15"/>
-      <c r="G60" s="15"/>
-      <c r="H60" s="16"/>
-      <c r="I60" s="10"/>
-      <c r="J60" s="10"/>
-    </row>
-    <row r="61" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="17">
+      <c r="B60" s="20"/>
+      <c r="C60" s="20"/>
+      <c r="D60" s="20"/>
+      <c r="E60" s="20"/>
+      <c r="F60" s="20"/>
+      <c r="G60" s="20"/>
+      <c r="H60" s="21"/>
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+    </row>
+    <row r="61" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="7">
         <v>1</v>
       </c>
-      <c r="B61" s="18" t="s">
+      <c r="B61" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C61" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D61" s="20" t="s">
+      <c r="C61" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D61" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E61" s="19" t="s">
+      <c r="E61" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F61" s="21" t="s">
+      <c r="F61" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G61" s="19" t="s">
+      <c r="G61" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H61" s="19" t="s">
+      <c r="H61" s="9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="17">
+    <row r="62" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="7">
         <v>2</v>
       </c>
-      <c r="B62" s="18" t="s">
+      <c r="B62" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C62" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D62" s="20" t="s">
+      <c r="C62" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D62" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E62" s="19" t="s">
+      <c r="E62" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="F62" s="19" t="s">
+      <c r="F62" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G62" s="19" t="s">
+      <c r="G62" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H62" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="17">
+      <c r="H62" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="7">
         <v>3</v>
       </c>
-      <c r="B63" s="18" t="s">
+      <c r="B63" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="C63" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D63" s="20" t="s">
+      <c r="C63" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D63" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="E63" s="19" t="s">
+      <c r="E63" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F63" s="19" t="s">
+      <c r="F63" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="G63" s="19" t="s">
+      <c r="G63" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H63" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="17">
+      <c r="H63" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="7">
         <v>4</v>
       </c>
-      <c r="B64" s="18" t="s">
+      <c r="B64" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="C64" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D64" s="20" t="s">
+      <c r="C64" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D64" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E64" s="19"/>
-      <c r="F64" s="19" t="s">
+      <c r="E64" s="9"/>
+      <c r="F64" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G64" s="19" t="s">
+      <c r="G64" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H64" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="17">
+      <c r="H64" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="7">
         <v>5</v>
       </c>
-      <c r="B65" s="18" t="s">
+      <c r="B65" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C65" s="19" t="s">
+      <c r="C65" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D65" s="20" t="s">
+      <c r="D65" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E65" s="19" t="s">
+      <c r="E65" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F65" s="19" t="s">
+      <c r="F65" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G65" s="19" t="s">
+      <c r="G65" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H65" s="19" t="s">
+      <c r="H65" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="14" t="s">
+      <c r="A66" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="B66" s="15"/>
-      <c r="C66" s="15"/>
-      <c r="D66" s="15"/>
-      <c r="E66" s="15"/>
-      <c r="F66" s="15"/>
-      <c r="G66" s="15"/>
-      <c r="H66" s="16"/>
-      <c r="I66" s="10"/>
-      <c r="J66" s="10"/>
-    </row>
-    <row r="67" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="17">
+      <c r="B66" s="20"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="21"/>
+      <c r="I66" s="3"/>
+      <c r="J66" s="3"/>
+    </row>
+    <row r="67" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="7">
         <v>1</v>
       </c>
-      <c r="B67" s="18" t="s">
+      <c r="B67" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="C67" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D67" s="20" t="s">
+      <c r="C67" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D67" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E67" s="19" t="s">
+      <c r="E67" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F67" s="19" t="s">
+      <c r="F67" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="G67" s="19" t="s">
+      <c r="G67" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H67" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J67" s="10" t="s">
+      <c r="H67" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J67" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="68" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="17">
+    <row r="68" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="7">
         <v>2</v>
       </c>
-      <c r="B68" s="18" t="s">
+      <c r="B68" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="C68" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D68" s="20" t="s">
+      <c r="C68" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D68" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E68" s="19" t="s">
+      <c r="E68" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F68" s="19" t="s">
+      <c r="F68" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="G68" s="19" t="s">
+      <c r="G68" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H68" s="19" t="s">
+      <c r="H68" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="14" t="s">
+      <c r="A69" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="B69" s="15"/>
-      <c r="C69" s="15"/>
-      <c r="D69" s="15"/>
-      <c r="E69" s="15"/>
-      <c r="F69" s="15"/>
-      <c r="G69" s="15"/>
-      <c r="H69" s="16"/>
-      <c r="I69" s="10"/>
-      <c r="J69" s="10"/>
-    </row>
-    <row r="70" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="17">
+      <c r="B69" s="20"/>
+      <c r="C69" s="20"/>
+      <c r="D69" s="20"/>
+      <c r="E69" s="20"/>
+      <c r="F69" s="20"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="21"/>
+      <c r="I69" s="3"/>
+      <c r="J69" s="3"/>
+    </row>
+    <row r="70" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="7">
         <v>1</v>
       </c>
-      <c r="B70" s="18" t="s">
+      <c r="B70" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="C70" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D70" s="20" t="s">
+      <c r="C70" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D70" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E70" s="19" t="s">
+      <c r="E70" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F70" s="19" t="s">
+      <c r="F70" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G70" s="19" t="s">
+      <c r="G70" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H70" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="17">
+      <c r="H70" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="7">
         <v>2</v>
       </c>
-      <c r="B71" s="18" t="s">
+      <c r="B71" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="C71" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D71" s="20" t="s">
+      <c r="C71" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D71" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E71" s="19" t="s">
+      <c r="E71" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F71" s="19" t="s">
+      <c r="F71" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G71" s="19" t="s">
+      <c r="G71" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H71" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="17">
+      <c r="H71" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="7">
         <v>3</v>
       </c>
-      <c r="B72" s="18" t="s">
+      <c r="B72" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="C72" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D72" s="20" t="s">
+      <c r="C72" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D72" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E72" s="19" t="s">
+      <c r="E72" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F72" s="19" t="s">
+      <c r="F72" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G72" s="19" t="s">
+      <c r="G72" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H72" s="19" t="s">
+      <c r="H72" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="14" t="s">
+      <c r="A73" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="B73" s="15"/>
-      <c r="C73" s="15"/>
-      <c r="D73" s="15"/>
-      <c r="E73" s="15"/>
-      <c r="F73" s="15"/>
-      <c r="G73" s="15"/>
-      <c r="H73" s="16"/>
-      <c r="I73" s="10"/>
-      <c r="J73" s="10"/>
-    </row>
-    <row r="74" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="17">
+      <c r="B73" s="20"/>
+      <c r="C73" s="20"/>
+      <c r="D73" s="20"/>
+      <c r="E73" s="20"/>
+      <c r="F73" s="20"/>
+      <c r="G73" s="20"/>
+      <c r="H73" s="21"/>
+      <c r="I73" s="3"/>
+      <c r="J73" s="3"/>
+    </row>
+    <row r="74" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="7">
         <v>1</v>
       </c>
-      <c r="B74" s="18" t="s">
+      <c r="B74" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="C74" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D74" s="20" t="s">
+      <c r="C74" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D74" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E74" s="19" t="s">
+      <c r="E74" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F74" s="19" t="s">
+      <c r="F74" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="G74" s="19" t="s">
+      <c r="G74" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H74" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="17">
+      <c r="H74" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="7">
         <v>2</v>
       </c>
-      <c r="B75" s="18" t="s">
+      <c r="B75" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="C75" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D75" s="20" t="s">
+      <c r="C75" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D75" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E75" s="19" t="s">
+      <c r="E75" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F75" s="19" t="s">
+      <c r="F75" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="G75" s="19" t="s">
+      <c r="G75" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H75" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="I75" s="10">
+      <c r="H75" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I75" s="3">
         <v>2023</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="17">
+    <row r="76" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="7">
         <v>3</v>
       </c>
-      <c r="B76" s="18" t="s">
+      <c r="B76" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="C76" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D76" s="20" t="s">
+      <c r="C76" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D76" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E76" s="19" t="s">
+      <c r="E76" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F76" s="19" t="s">
+      <c r="F76" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G76" s="19" t="s">
+      <c r="G76" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H76" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="17">
+      <c r="H76" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="7">
         <v>4</v>
       </c>
-      <c r="B77" s="18" t="s">
+      <c r="B77" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="C77" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D77" s="20" t="s">
+      <c r="C77" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D77" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E77" s="19" t="s">
+      <c r="E77" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F77" s="19" t="s">
+      <c r="F77" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G77" s="19" t="s">
+      <c r="G77" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="H77" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="17">
+      <c r="H77" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="7">
         <v>5</v>
       </c>
-      <c r="B78" s="18" t="s">
+      <c r="B78" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="C78" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D78" s="20" t="s">
+      <c r="C78" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D78" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E78" s="19" t="s">
+      <c r="E78" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F78" s="19" t="s">
+      <c r="F78" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G78" s="19" t="s">
+      <c r="G78" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H78" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="17">
+      <c r="H78" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="7">
         <v>6</v>
       </c>
-      <c r="B79" s="18" t="s">
+      <c r="B79" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="C79" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D79" s="20" t="s">
+      <c r="C79" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D79" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E79" s="19" t="s">
+      <c r="E79" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F79" s="19" t="s">
+      <c r="F79" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G79" s="19" t="s">
+      <c r="G79" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H79" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="17">
+      <c r="H79" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="7">
         <v>7</v>
       </c>
-      <c r="B80" s="18" t="s">
+      <c r="B80" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="C80" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D80" s="20" t="s">
+      <c r="C80" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D80" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E80" s="19" t="s">
+      <c r="E80" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F80" s="19" t="s">
+      <c r="F80" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="G80" s="19" t="s">
+      <c r="G80" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H80" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="81" spans="1:8" s="10" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="17">
+      <c r="H80" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" s="3" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="7">
         <v>8</v>
       </c>
-      <c r="B81" s="18" t="s">
+      <c r="B81" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="C81" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D81" s="20" t="s">
+      <c r="C81" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D81" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E81" s="19" t="s">
+      <c r="E81" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F81" s="19" t="s">
+      <c r="F81" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="G81" s="19" t="s">
+      <c r="G81" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="H81" s="19"/>
+      <c r="H81" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A66:H66"/>
     <mergeCell ref="A69:H69"/>
     <mergeCell ref="A73:H73"/>
@@ -3637,18 +3649,6 @@
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A54:H54"/>
     <mergeCell ref="A60:H60"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:D6"/>
   </mergeCells>
   <pageMargins left="0.27" right="0.2" top="0.16" bottom="0.12" header="0.18" footer="0.12"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>